<commit_message>
Add Vendor category to sign inventory workbook
Category dropdown now offers Sponsor/Vendor/Operations, the name column
covers vendors as well, the Summary sheet tallies vendor signs
separately, and the blank fill-in section grew to 40 rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vs8vaQzMdxg2Fp1ZjjtAuw
</commit_message>
<xml_diff>
--- a/marketing/sign-inventory.xlsx
+++ b/marketing/sign-inventory.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Sign Inventory'!$A$4:$K$65</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Sign Inventory'!$A$4:$K$75</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="91">
   <si>
     <t xml:space="preserve">HOLMDALE PRO RODEO — SIGN INVENTORY</t>
   </si>
   <si>
-    <t xml:space="preserve">HOW TO USE: Fill in the YELLOW cells during your walk-through. One row per sign (or per batch of identical signs — use Qty). Category, Size, Material and Condition have dropdowns, but you can type your own value. For sponsor signs, put the sponsor's name in column D. Row 5 is an EXAMPLE only — overwrite or delete it.</t>
+    <t xml:space="preserve">HOW TO USE: Fill in the YELLOW cells during your walk-through. One row per sign (or per batch of identical signs — use Qty). Category, Size, Material and Condition have dropdowns, but you can type your own value. For sponsor or vendor signs, put the sponsor's/vendor's name in column D. Row 5 is an EXAMPLE only — overwrite or delete it.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">Category</t>
   </si>
   <si>
-    <t xml:space="preserve">Sponsor (if applicable)</t>
+    <t xml:space="preserve">Sponsor / Vendor (if applicable)</t>
   </si>
   <si>
     <t xml:space="preserve">Size</t>
@@ -198,6 +198,9 @@
     <t xml:space="preserve">New</t>
   </si>
   <si>
+    <t xml:space="preserve">Vendor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vinyl banner</t>
   </si>
   <si>
@@ -280,6 +283,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sponsor signs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendor signs</t>
   </si>
   <si>
     <t xml:space="preserve">Operations signs</t>
@@ -844,7 +850,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2101,26 +2107,186 @@
       <c r="J65" s="9"/>
       <c r="K65" s="9"/>
     </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7" t="str">
+        <f aca="false">IF(B66="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B66" s="9"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="9"/>
+      <c r="F66" s="9"/>
+      <c r="G66" s="10"/>
+      <c r="H66" s="9"/>
+      <c r="I66" s="9"/>
+      <c r="J66" s="9"/>
+      <c r="K66" s="9"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="str">
+        <f aca="false">IF(B67="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="9"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="9"/>
+      <c r="I67" s="9"/>
+      <c r="J67" s="9"/>
+      <c r="K67" s="9"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7" t="str">
+        <f aca="false">IF(B68="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="9"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="9"/>
+      <c r="I68" s="9"/>
+      <c r="J68" s="9"/>
+      <c r="K68" s="9"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7" t="str">
+        <f aca="false">IF(B69="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9"/>
+      <c r="G69" s="10"/>
+      <c r="H69" s="9"/>
+      <c r="I69" s="9"/>
+      <c r="J69" s="9"/>
+      <c r="K69" s="9"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="7" t="str">
+        <f aca="false">IF(B70="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="9"/>
+      <c r="F70" s="9"/>
+      <c r="G70" s="10"/>
+      <c r="H70" s="9"/>
+      <c r="I70" s="9"/>
+      <c r="J70" s="9"/>
+      <c r="K70" s="9"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="7" t="str">
+        <f aca="false">IF(B71="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9"/>
+      <c r="G71" s="10"/>
+      <c r="H71" s="9"/>
+      <c r="I71" s="9"/>
+      <c r="J71" s="9"/>
+      <c r="K71" s="9"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="7" t="str">
+        <f aca="false">IF(B72="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9"/>
+      <c r="F72" s="9"/>
+      <c r="G72" s="10"/>
+      <c r="H72" s="9"/>
+      <c r="I72" s="9"/>
+      <c r="J72" s="9"/>
+      <c r="K72" s="9"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="7" t="str">
+        <f aca="false">IF(B73="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+      <c r="F73" s="9"/>
+      <c r="G73" s="10"/>
+      <c r="H73" s="9"/>
+      <c r="I73" s="9"/>
+      <c r="J73" s="9"/>
+      <c r="K73" s="9"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="7" t="str">
+        <f aca="false">IF(B74="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B74" s="9"/>
+      <c r="C74" s="9"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="9"/>
+      <c r="G74" s="10"/>
+      <c r="H74" s="9"/>
+      <c r="I74" s="9"/>
+      <c r="J74" s="9"/>
+      <c r="K74" s="9"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="7" t="str">
+        <f aca="false">IF(B75="","",ROW()-4)</f>
+        <v/>
+      </c>
+      <c r="B75" s="9"/>
+      <c r="C75" s="9"/>
+      <c r="D75" s="9"/>
+      <c r="E75" s="9"/>
+      <c r="F75" s="9"/>
+      <c r="G75" s="10"/>
+      <c r="H75" s="9"/>
+      <c r="I75" s="9"/>
+      <c r="J75" s="9"/>
+      <c r="K75" s="9"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K65"/>
+  <autoFilter ref="A4:K75"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C65" type="list">
-      <formula1>Lists!$A$2:$A$3</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C75" type="list">
+      <formula1>Lists!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E65" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E75" type="list">
       <formula1>Lists!$C$2:$C$12</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F65" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F75" type="list">
       <formula1>Lists!$B$2:$B$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H65" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H75" type="list">
       <formula1>Lists!$D$2:$D$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2180,54 +2346,57 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>23</v>
+      </c>
       <c r="B4" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>16</v>
@@ -2235,39 +2404,39 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2286,7 +2455,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -2296,167 +2465,167 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B5" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$B$5:$B$65,"&lt;&gt;")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$B$5:$B$75,"&lt;&gt;")</f>
         <v>31</v>
       </c>
       <c r="C5" s="17" t="n">
-        <f aca="false">SUM('Sign Inventory'!$G$5:$G$65)</f>
+        <f aca="false">SUM('Sign Inventory'!$G$5:$G$75)</f>
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B6" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$C$5:$C$65,"Sponsor")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$C$5:$C$75,"Sponsor")</f>
         <v>1</v>
       </c>
       <c r="C6" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$C$5:$C$65,"Sponsor")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$C$5:$C$75,"Sponsor")</f>
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B7" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$C$5:$C$65,"Operations")</f>
-        <v>30</v>
+        <f aca="false">COUNTIF('Sign Inventory'!$C$5:$C$75,"Vendor")</f>
+        <v>0</v>
       </c>
       <c r="C7" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$C$5:$C$65,"Operations")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$C$5:$C$75,"Vendor")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B8" s="17" t="n">
-        <f aca="false">COUNTIFS('Sign Inventory'!$B$5:$B$65,"&lt;&gt;",'Sign Inventory'!$C$5:$C$65,"")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$C$5:$C$75,"Operations")</f>
+        <v>30</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$C$5:$C$75,"Operations")</f>
         <v>0</v>
       </c>
-      <c r="C8" s="17"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
+      <c r="A9" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <f aca="false">COUNTIFS('Sign Inventory'!$B$5:$B$75,"&lt;&gt;",'Sign Inventory'!$C$5:$C$75,"")</f>
+        <v>0</v>
+      </c>
       <c r="C9" s="17"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="15" t="s">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="15" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Coroplast (corrugated plastic)")</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Coroplast (corrugated plastic)")</f>
-        <v>2</v>
+      <c r="C11" s="15" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="B12" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Vinyl banner")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Coroplast (corrugated plastic)")</f>
+        <v>1</v>
       </c>
       <c r="C12" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Vinyl banner")</f>
-        <v>0</v>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Coroplast (corrugated plastic)")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Mesh banner")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Vinyl banner")</f>
         <v>0</v>
       </c>
       <c r="C13" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Mesh banner")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Vinyl banner")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B14" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Aluminum / metal")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Mesh banner")</f>
         <v>0</v>
       </c>
       <c r="C14" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Aluminum / metal")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Mesh banner")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B15" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Plywood (painted)")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Aluminum / metal")</f>
         <v>0</v>
       </c>
       <c r="C15" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Plywood (painted)")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Aluminum / metal")</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B16" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"PVC / Sintra board")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Plywood (painted)")</f>
         <v>0</v>
       </c>
       <c r="C16" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"PVC / Sintra board")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Plywood (painted)")</f>
         <v>0</v>
       </c>
     </row>
@@ -2465,116 +2634,129 @@
         <v>69</v>
       </c>
       <c r="B17" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Fabric flag")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"PVC / Sintra board")</f>
         <v>0</v>
       </c>
       <c r="C17" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Fabric flag")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"PVC / Sintra board")</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B18" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Magnetic")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Fabric flag")</f>
         <v>0</v>
       </c>
       <c r="C18" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Magnetic")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Fabric flag")</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Cardboard / paper")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Magnetic")</f>
         <v>0</v>
       </c>
       <c r="C19" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Cardboard / paper")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Magnetic")</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B20" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$65,"Other")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Cardboard / paper")</f>
         <v>0</v>
       </c>
       <c r="C20" s="17" t="n">
-        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$65,'Sign Inventory'!$F$5:$F$65,"Other")</f>
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Cardboard / paper")</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
+      <c r="A21" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="17" t="n">
+        <f aca="false">COUNTIF('Sign Inventory'!$F$5:$F$75,"Other")</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <f aca="false">SUMIFS('Sign Inventory'!$G$5:$G$75,'Sign Inventory'!$F$5:$F$75,"Other")</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C22" s="15"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B23" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$65,"New")</f>
-        <v>0</v>
-      </c>
-      <c r="C23" s="17"/>
+      <c r="A23" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="B24" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$65,"Good")</f>
-        <v>1</v>
+        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$75,"New")</f>
+        <v>0</v>
       </c>
       <c r="C24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="B25" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$65,"Fair")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$75,"Good")</f>
+        <v>1</v>
       </c>
       <c r="C25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B26" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$65,"Needs repair")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$75,"Fair")</f>
         <v>0</v>
       </c>
       <c r="C26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B27" s="17" t="n">
-        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$65,"Replace")</f>
+        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$75,"Needs repair")</f>
         <v>0</v>
       </c>
       <c r="C27" s="17"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="17" t="n">
+        <f aca="false">COUNTIF('Sign Inventory'!$H$5:$H$75,"Replace")</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>